<commit_message>
fix: show empty professor cells as blank in Asignaturas sheet
</commit_message>
<xml_diff>
--- a/ejemplos-generados/gestion-departamento.xlsx
+++ b/ejemplos-generados/gestion-departamento.xlsx
@@ -2236,7 +2236,7 @@
         <v>32</v>
       </c>
       <c r="D5" s="6">
-        <f>'Asignación'!F4</f>
+        <f>IF('Asignación'!F4="","",'Asignación'!F4)</f>
         <v/>
       </c>
       <c r="E5" s="7">
@@ -2257,7 +2257,7 @@
         <v>32</v>
       </c>
       <c r="D6" s="6">
-        <f>'Asignación'!F5</f>
+        <f>IF('Asignación'!F5="","",'Asignación'!F5)</f>
         <v/>
       </c>
       <c r="E6" s="7">
@@ -2278,7 +2278,7 @@
         <v>32</v>
       </c>
       <c r="D7" s="9">
-        <f>'Asignación'!F6</f>
+        <f>IF('Asignación'!F6="","",'Asignación'!F6)</f>
         <v/>
       </c>
       <c r="E7" s="10">
@@ -2340,7 +2340,7 @@
         <v>32</v>
       </c>
       <c r="D11" s="6">
-        <f>'Asignación'!F7</f>
+        <f>IF('Asignación'!F7="","",'Asignación'!F7)</f>
         <v/>
       </c>
       <c r="E11" s="7">
@@ -2361,7 +2361,7 @@
         <v>32</v>
       </c>
       <c r="D12" s="9">
-        <f>'Asignación'!F8</f>
+        <f>IF('Asignación'!F8="","",'Asignación'!F8)</f>
         <v/>
       </c>
       <c r="E12" s="10">
@@ -2423,7 +2423,7 @@
         <v>48</v>
       </c>
       <c r="D16" s="6">
-        <f>'Asignación'!F9</f>
+        <f>IF('Asignación'!F9="","",'Asignación'!F9)</f>
         <v/>
       </c>
       <c r="E16" s="7">
@@ -2444,7 +2444,7 @@
         <v>32</v>
       </c>
       <c r="D17" s="6">
-        <f>'Asignación'!F10</f>
+        <f>IF('Asignación'!F10="","",'Asignación'!F10)</f>
         <v/>
       </c>
       <c r="E17" s="7">
@@ -2465,7 +2465,7 @@
         <v>32</v>
       </c>
       <c r="D18" s="6">
-        <f>'Asignación'!F11</f>
+        <f>IF('Asignación'!F11="","",'Asignación'!F11)</f>
         <v/>
       </c>
       <c r="E18" s="7">
@@ -2486,7 +2486,7 @@
         <v>32</v>
       </c>
       <c r="D19" s="9">
-        <f>'Asignación'!F12</f>
+        <f>IF('Asignación'!F12="","",'Asignación'!F12)</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -2548,7 +2548,7 @@
         <v>16</v>
       </c>
       <c r="D23" s="9">
-        <f>'Asignación'!F13</f>
+        <f>IF('Asignación'!F13="","",'Asignación'!F13)</f>
         <v/>
       </c>
       <c r="E23" s="10">

</xml_diff>

<commit_message>
fix: size formula columns from the values they can show
</commit_message>
<xml_diff>
--- a/ejemplos-generados/gestion-departamento.xlsx
+++ b/ejemplos-generados/gestion-departamento.xlsx
@@ -618,7 +618,7 @@
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -997,7 +997,7 @@
   <dimension ref="A1:D68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="43" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -2171,8 +2171,8 @@
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
feat: apply row-height padding to Profesores and Asignaturas sheets
</commit_message>
<xml_diff>
--- a/ejemplos-generados/gestion-departamento.xlsx
+++ b/ejemplos-generados/gestion-departamento.xlsx
@@ -1011,7 +1011,7 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3">
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Id</t>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>PIAD</t>
@@ -1053,7 +1053,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Asignatura</t>
@@ -1075,7 +1075,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="5">
         <f>IFERROR(VLOOKUP("PIAD#1",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1093,7 +1093,7 @@
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5">
         <f>IFERROR(VLOOKUP("PIAD#2",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1111,7 +1111,7 @@
         <v/>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="22" customHeight="1">
       <c r="A8" s="5">
         <f>IFERROR(VLOOKUP("PIAD#3",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1129,7 +1129,7 @@
         <v/>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="5">
         <f>IFERROR(VLOOKUP("PIAD#4",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1147,7 +1147,7 @@
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="5">
         <f>IFERROR(VLOOKUP("PIAD#5",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1165,7 +1165,7 @@
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="5">
         <f>IFERROR(VLOOKUP("PIAD#6",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1183,7 +1183,7 @@
         <v/>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="22" customHeight="1">
       <c r="A12" s="5">
         <f>IFERROR(VLOOKUP("PIAD#7",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1201,7 +1201,7 @@
         <v/>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="22" customHeight="1">
       <c r="A13" s="5">
         <f>IF(COUNTIF('Asignación'!$F$4:$F$13,"PIAD")&gt;8,"(+"&amp;(COUNTIF('Asignación'!$F$4:$F$13,"PIAD")-8+1)&amp;" más)",IFERROR(VLOOKUP("PIAD#8",CargaPorProfesor,2,0),""))</f>
         <v/>
@@ -1219,7 +1219,7 @@
         <v/>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="22" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
@@ -1232,8 +1232,8 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16">
+    <row r="15" ht="22" customHeight="1"/>
+    <row r="16" ht="22" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Id</t>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>MARA</t>
@@ -1275,7 +1275,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="22" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Asignatura</t>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="22" customHeight="1">
       <c r="A19" s="5">
         <f>IFERROR(VLOOKUP("MARA#1",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1315,7 +1315,7 @@
         <v/>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="22" customHeight="1">
       <c r="A20" s="5">
         <f>IFERROR(VLOOKUP("MARA#2",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1333,7 +1333,7 @@
         <v/>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="22" customHeight="1">
       <c r="A21" s="5">
         <f>IFERROR(VLOOKUP("MARA#3",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1351,7 +1351,7 @@
         <v/>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="22" customHeight="1">
       <c r="A22" s="5">
         <f>IFERROR(VLOOKUP("MARA#4",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1369,7 +1369,7 @@
         <v/>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="5">
         <f>IFERROR(VLOOKUP("MARA#5",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="22" customHeight="1">
       <c r="A24" s="5">
         <f>IFERROR(VLOOKUP("MARA#6",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1405,7 +1405,7 @@
         <v/>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="22" customHeight="1">
       <c r="A25" s="5">
         <f>IFERROR(VLOOKUP("MARA#7",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1423,7 +1423,7 @@
         <v/>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="22" customHeight="1">
       <c r="A26" s="5">
         <f>IF(COUNTIF('Asignación'!$F$4:$F$13,"MARA")&gt;8,"(+"&amp;(COUNTIF('Asignación'!$F$4:$F$13,"MARA")-8+1)&amp;" más)",IFERROR(VLOOKUP("MARA#8",CargaPorProfesor,2,0),""))</f>
         <v/>
@@ -1441,7 +1441,7 @@
         <v/>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="22" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
@@ -1454,8 +1454,8 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29">
+    <row r="28" ht="22" customHeight="1"/>
+    <row r="29" ht="22" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Id</t>
@@ -1477,7 +1477,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="22" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>LGOM</t>
@@ -1497,7 +1497,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="22" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
           <t>Asignatura</t>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="22" customHeight="1">
       <c r="A32" s="5">
         <f>IFERROR(VLOOKUP("LGOM#1",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1537,7 +1537,7 @@
         <v/>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="22" customHeight="1">
       <c r="A33" s="5">
         <f>IFERROR(VLOOKUP("LGOM#2",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1555,7 +1555,7 @@
         <v/>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="22" customHeight="1">
       <c r="A34" s="5">
         <f>IFERROR(VLOOKUP("LGOM#3",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1573,7 +1573,7 @@
         <v/>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="22" customHeight="1">
       <c r="A35" s="5">
         <f>IFERROR(VLOOKUP("LGOM#4",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1591,7 +1591,7 @@
         <v/>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="22" customHeight="1">
       <c r="A36" s="5">
         <f>IFERROR(VLOOKUP("LGOM#5",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1609,7 +1609,7 @@
         <v/>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="22" customHeight="1">
       <c r="A37" s="5">
         <f>IFERROR(VLOOKUP("LGOM#6",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1627,7 +1627,7 @@
         <v/>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="22" customHeight="1">
       <c r="A38" s="5">
         <f>IFERROR(VLOOKUP("LGOM#7",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1645,7 +1645,7 @@
         <v/>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="22" customHeight="1">
       <c r="A39" s="5">
         <f>IF(COUNTIF('Asignación'!$F$4:$F$13,"LGOM")&gt;8,"(+"&amp;(COUNTIF('Asignación'!$F$4:$F$13,"LGOM")-8+1)&amp;" más)",IFERROR(VLOOKUP("LGOM#8",CargaPorProfesor,2,0),""))</f>
         <v/>
@@ -1663,7 +1663,7 @@
         <v/>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="22" customHeight="1">
       <c r="A40" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
@@ -1676,8 +1676,8 @@
         <v/>
       </c>
     </row>
-    <row r="41"/>
-    <row r="42">
+    <row r="41" ht="22" customHeight="1"/>
+    <row r="42" ht="22" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Id</t>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="22" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
           <t>ANSU</t>
@@ -1719,7 +1719,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="22" customHeight="1">
       <c r="A44" s="13" t="inlineStr">
         <is>
           <t>Asignatura</t>
@@ -1741,7 +1741,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="22" customHeight="1">
       <c r="A45" s="5">
         <f>IFERROR(VLOOKUP("ANSU#1",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1759,7 +1759,7 @@
         <v/>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="22" customHeight="1">
       <c r="A46" s="5">
         <f>IFERROR(VLOOKUP("ANSU#2",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1777,7 +1777,7 @@
         <v/>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="22" customHeight="1">
       <c r="A47" s="5">
         <f>IFERROR(VLOOKUP("ANSU#3",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1795,7 +1795,7 @@
         <v/>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="22" customHeight="1">
       <c r="A48" s="5">
         <f>IFERROR(VLOOKUP("ANSU#4",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1813,7 +1813,7 @@
         <v/>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="22" customHeight="1">
       <c r="A49" s="5">
         <f>IFERROR(VLOOKUP("ANSU#5",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1831,7 +1831,7 @@
         <v/>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="22" customHeight="1">
       <c r="A50" s="5">
         <f>IFERROR(VLOOKUP("ANSU#6",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1849,7 +1849,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="22" customHeight="1">
       <c r="A51" s="5">
         <f>IFERROR(VLOOKUP("ANSU#7",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1867,7 +1867,7 @@
         <v/>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="22" customHeight="1">
       <c r="A52" s="5">
         <f>IF(COUNTIF('Asignación'!$F$4:$F$13,"ANSU")&gt;8,"(+"&amp;(COUNTIF('Asignación'!$F$4:$F$13,"ANSU")-8+1)&amp;" más)",IFERROR(VLOOKUP("ANSU#8",CargaPorProfesor,2,0),""))</f>
         <v/>
@@ -1885,7 +1885,7 @@
         <v/>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="22" customHeight="1">
       <c r="A53" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
@@ -1898,8 +1898,8 @@
         <v/>
       </c>
     </row>
-    <row r="54"/>
-    <row r="55">
+    <row r="54" ht="22" customHeight="1"/>
+    <row r="55" ht="22" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Id</t>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="22" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
           <t>RTOR</t>
@@ -1941,7 +1941,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="22" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
           <t>Asignatura</t>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="22" customHeight="1">
       <c r="A58" s="5">
         <f>IFERROR(VLOOKUP("RTOR#1",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1981,7 +1981,7 @@
         <v/>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="22" customHeight="1">
       <c r="A59" s="5">
         <f>IFERROR(VLOOKUP("RTOR#2",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -1999,7 +1999,7 @@
         <v/>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="22" customHeight="1">
       <c r="A60" s="5">
         <f>IFERROR(VLOOKUP("RTOR#3",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -2017,7 +2017,7 @@
         <v/>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="22" customHeight="1">
       <c r="A61" s="5">
         <f>IFERROR(VLOOKUP("RTOR#4",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -2035,7 +2035,7 @@
         <v/>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="22" customHeight="1">
       <c r="A62" s="5">
         <f>IFERROR(VLOOKUP("RTOR#5",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -2053,7 +2053,7 @@
         <v/>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="22" customHeight="1">
       <c r="A63" s="5">
         <f>IFERROR(VLOOKUP("RTOR#6",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -2071,7 +2071,7 @@
         <v/>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="22" customHeight="1">
       <c r="A64" s="5">
         <f>IFERROR(VLOOKUP("RTOR#7",CargaPorProfesor,2,0),"")</f>
         <v/>
@@ -2089,7 +2089,7 @@
         <v/>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="22" customHeight="1">
       <c r="A65" s="5">
         <f>IF(COUNTIF('Asignación'!$F$4:$F$13,"RTOR")&gt;8,"(+"&amp;(COUNTIF('Asignación'!$F$4:$F$13,"RTOR")-8+1)&amp;" más)",IFERROR(VLOOKUP("RTOR#8",CargaPorProfesor,2,0),""))</f>
         <v/>
@@ -2107,7 +2107,7 @@
         <v/>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="22" customHeight="1">
       <c r="A66" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
@@ -2183,7 +2183,7 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3">
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Estadística (CC) — Ciencia de la Computación</t>
@@ -2194,7 +2194,7 @@
       <c r="D3" s="19" t="n"/>
       <c r="E3" s="20" t="n"/>
     </row>
-    <row r="4">
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Conf</t>
@@ -2244,7 +2244,7 @@
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>CP</t>
@@ -2265,7 +2265,7 @@
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>CP</t>
@@ -2286,8 +2286,8 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9">
+    <row r="8" ht="22" customHeight="1"/>
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Estadística (Mat) — Matemática</t>
@@ -2298,7 +2298,7 @@
       <c r="D9" s="19" t="n"/>
       <c r="E9" s="20" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -2325,7 +2325,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Conf</t>
@@ -2348,7 +2348,7 @@
         <v/>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>CP</t>
@@ -2369,8 +2369,8 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
+    <row r="13" ht="22" customHeight="1"/>
+    <row r="14" ht="22" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Análisis Numérico (CD) — Ciencia de Datos</t>
@@ -2381,7 +2381,7 @@
       <c r="D14" s="19" t="n"/>
       <c r="E14" s="20" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -2408,7 +2408,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="22" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Conf</t>
@@ -2431,7 +2431,7 @@
         <v/>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>CP</t>
@@ -2452,7 +2452,7 @@
         <v/>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="22" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>CP</t>
@@ -2473,7 +2473,7 @@
         <v/>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="22" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>CP</t>
@@ -2494,8 +2494,8 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
+    <row r="20" ht="22" customHeight="1"/>
+    <row r="21" ht="22" customHeight="1">
       <c r="A21" s="18" t="inlineStr">
         <is>
           <t>Seminario de Matemática — Matemática</t>
@@ -2506,7 +2506,7 @@
       <c r="D21" s="19" t="n"/>
       <c r="E21" s="20" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="22" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Conf</t>
@@ -2556,7 +2556,7 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
+    <row r="24" ht="22" customHeight="1"/>
     <row r="25"/>
     <row r="26">
       <c r="A26" s="21" t="n"/>

</xml_diff>

<commit_message>
feat: draw thick separators between asignaturas in Asignacion sheet
</commit_message>
<xml_diff>
--- a/ejemplos-generados/gestion-departamento.xlsx
+++ b/ejemplos-generados/gestion-departamento.xlsx
@@ -80,7 +80,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -142,11 +142,29 @@
       <top style="thin"/>
       <bottom style="medium"/>
     </border>
+    <border>
+      <left style="medium"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thick"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thick"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="thick"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -165,6 +183,15 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -725,29 +752,29 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Estadística (CC)</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Ciencia de la Computación</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="7">
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="10">
         <f>IF(F6="","",IFERROR(VLOOKUP(F6,ProfesoresTabla,2,0),"(desconocido)"))</f>
         <v/>
       </c>
@@ -783,29 +810,29 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Estadística (Mat)</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Matemática</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="7">
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="10">
         <f>IF(F8="","",IFERROR(VLOOKUP(F8,ProfesoresTabla,2,0),"(desconocido)"))</f>
         <v/>
       </c>
@@ -897,65 +924,65 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Análisis Numérico (CD)</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Ciencia de Datos</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="7">
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="10">
         <f>IF(F12="","",IFERROR(VLOOKUP(F12,ProfesoresTabla,2,0),"(desconocido)"))</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Seminario de Matemática</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Matemática</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Conf</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="10">
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="13">
         <f>IF(F13="","",IFERROR(VLOOKUP(F13,ProfesoresTabla,2,0),"(desconocido)"))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
+      <c r="A15" s="14" t="n"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>Falta asignar profesor</t>
@@ -963,7 +990,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
+      <c r="A16" s="15" t="n"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Profesor fuera de la lista</t>
@@ -1054,22 +1081,22 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Asignatura</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
@@ -1220,14 +1247,14 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="10">
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="13">
         <f>SUMIF('Asignación'!$F$4:$F$13,"PIAD",'Asignación'!$E$4:$E$13)</f>
         <v/>
       </c>
@@ -1276,22 +1303,22 @@
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Asignatura</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
@@ -1442,14 +1469,14 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="10">
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="13">
         <f>SUMIF('Asignación'!$F$4:$F$13,"MARA",'Asignación'!$E$4:$E$13)</f>
         <v/>
       </c>
@@ -1498,22 +1525,22 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Asignatura</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="D31" s="18" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
@@ -1664,14 +1691,14 @@
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B40" s="9" t="n"/>
-      <c r="C40" s="9" t="n"/>
-      <c r="D40" s="10">
+      <c r="B40" s="12" t="n"/>
+      <c r="C40" s="12" t="n"/>
+      <c r="D40" s="13">
         <f>SUMIF('Asignación'!$F$4:$F$13,"LGOM",'Asignación'!$E$4:$E$13)</f>
         <v/>
       </c>
@@ -1720,22 +1747,22 @@
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>Asignatura</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B44" s="17" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C44" s="14" t="inlineStr">
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="D44" s="18" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
@@ -1886,14 +1913,14 @@
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="16" t="inlineStr">
+      <c r="A53" s="19" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B53" s="9" t="n"/>
-      <c r="C53" s="9" t="n"/>
-      <c r="D53" s="10">
+      <c r="B53" s="12" t="n"/>
+      <c r="C53" s="12" t="n"/>
+      <c r="D53" s="13">
         <f>SUMIF('Asignación'!$F$4:$F$13,"ANSU",'Asignación'!$E$4:$E$13)</f>
         <v/>
       </c>
@@ -1942,22 +1969,22 @@
       </c>
     </row>
     <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="13" t="inlineStr">
+      <c r="A57" s="16" t="inlineStr">
         <is>
           <t>Asignatura</t>
         </is>
       </c>
-      <c r="B57" s="14" t="inlineStr">
+      <c r="B57" s="17" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C57" s="14" t="inlineStr">
+      <c r="C57" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="D57" s="15" t="inlineStr">
+      <c r="D57" s="18" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
@@ -2108,21 +2135,21 @@
       </c>
     </row>
     <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="16" t="inlineStr">
+      <c r="A66" s="19" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B66" s="9" t="n"/>
-      <c r="C66" s="9" t="n"/>
-      <c r="D66" s="10">
+      <c r="B66" s="12" t="n"/>
+      <c r="C66" s="12" t="n"/>
+      <c r="D66" s="13">
         <f>SUMIF('Asignación'!$F$4:$F$13,"RTOR",'Asignación'!$E$4:$E$13)</f>
         <v/>
       </c>
     </row>
     <row r="67"/>
     <row r="68">
-      <c r="A68" s="17" t="n"/>
+      <c r="A68" s="20" t="n"/>
       <c r="B68" t="inlineStr">
         <is>
           <t>Profesor por encima de su tope de horas</t>
@@ -2184,38 +2211,38 @@
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Estadística (CC) — Ciencia de la Computación</t>
         </is>
       </c>
-      <c r="B3" s="19" t="n"/>
-      <c r="C3" s="19" t="n"/>
-      <c r="D3" s="19" t="n"/>
-      <c r="E3" s="20" t="n"/>
+      <c r="B3" s="22" t="n"/>
+      <c r="C3" s="22" t="n"/>
+      <c r="D3" s="22" t="n"/>
+      <c r="E3" s="23" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>Profesor</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
@@ -2266,60 +2293,60 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="12">
         <f>IF('Asignación'!F6="","",'Asignación'!F6)</f>
         <v/>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="13">
         <f>'Asignación'!G6</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1"/>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Estadística (Mat) — Matemática</t>
         </is>
       </c>
-      <c r="B9" s="19" t="n"/>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="20" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="23" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>Profesor</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
@@ -2349,60 +2376,60 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="12">
         <f>IF('Asignación'!F8="","",'Asignación'!F8)</f>
         <v/>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="13">
         <f>'Asignación'!G8</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>Análisis Numérico (CD) — Ciencia de Datos</t>
         </is>
       </c>
-      <c r="B14" s="19" t="n"/>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
-      <c r="E14" s="20" t="n"/>
+      <c r="B14" s="22" t="n"/>
+      <c r="C14" s="22" t="n"/>
+      <c r="D14" s="22" t="n"/>
+      <c r="E14" s="23" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>Profesor</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
@@ -2474,84 +2501,84 @@
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n">
+      <c r="B19" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="12">
         <f>IF('Asignación'!F12="","",'Asignación'!F12)</f>
         <v/>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="13">
         <f>'Asignación'!G12</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Seminario de Matemática — Matemática</t>
         </is>
       </c>
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-      <c r="E21" s="20" t="n"/>
+      <c r="B21" s="22" t="n"/>
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="23" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>Horas</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>Profesor</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Conf</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="12">
         <f>IF('Asignación'!F13="","",'Asignación'!F13)</f>
         <v/>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="13">
         <f>'Asignación'!G13</f>
         <v/>
       </c>
@@ -2559,7 +2586,7 @@
     <row r="24" ht="22" customHeight="1"/>
     <row r="25"/>
     <row r="26">
-      <c r="A26" s="21" t="n"/>
+      <c r="A26" s="24" t="n"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>Asignatura completa (todo asignado)</t>
@@ -2567,7 +2594,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="n"/>
+      <c r="A27" s="25" t="n"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>Asignatura incompleta (faltan profesores)</t>

</xml_diff>